<commit_message>
Analisi: rettifiche della revisione indipendente sui modelli di Arluno e Basiano
- Arluno: gli arretrati condominiali (9.350) sono le detrazioni della
  perizia, non insoluti accertati: ora IPOTESI prudenziale, con lo stato
  debitorio da chiedere all'amministratore;
- Arluno: la cauzione del 10% e' scritta nell'avviso (sezione F): dato,
  non ipotesi; fra gli avvisi elettrodotto e impianti senza certificazioni
  (APE F); secondo avviso;
- Basiano: edificio di interesse storico-culturale nel PGT, che pesa sui
  lavori di copertura e facciate; 'IV esperimento' con la sua fonte
  (nome dell'allegato PVP);
- README: per Arluno l'uscita necessaria all'offerta minima (1.781 EUR/mq),
  non quella al prezzo base.
Prezzi massimi e margini invariati; check_workbook: 0 errori.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014uQ3c5E7LnkYiWheXFjKjz
</commit_message>
<xml_diff>
--- a/analisi/arluno-carso-fix-and-flip.xlsx
+++ b/analisi/arluno-carso-fix-and-flip.xlsx
@@ -59,8 +59,8 @@
     <definedName name="Arv">'Inputs'!$B$52</definedName>
     <definedName name="LavoriTot">'Inputs'!$B$53</definedName>
     <definedName name="TassoMese">'Inputs'!$B$54</definedName>
-    <definedName name="ErroriTot">'Checks'!$B$21</definedName>
-    <definedName name="AvvisiTot">'Checks'!$B$22</definedName>
+    <definedName name="ErroriTot">'Checks'!$B$22</definedName>
+    <definedName name="AvvisiTot">'Checks'!$B$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -540,7 +540,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Via Del Carso 2-4-6, Arluno (MI), zona OMI B1. Trilocale A/3 al 2 piano senza ascensore, cantina e box 21 mq; edificio anni '70. RGE 1138/2025, asta 02/12/2026.</t>
+          <t>Via Del Carso 2-4-6, Arluno (MI), zona OMI B1. Trilocale A/3 al 2 piano senza ascensore, cantina e box 21 mq; edificio anni '70. RGE 1138/2025, secondo avviso (gia' deserto una volta), asta 02/12/2026.</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Da confermare prima di offrire: stato interno al sopralluogo, tempi di liberazione, assemblee condominiali recenti, regime fiscale, percentuale della cauzione.</t>
+          <t>Da confermare prima di offrire: stato debitorio condominiale dall'amministratore, stato interno e impianti al sopralluogo, vincoli dell'elettrodotto, tempi di liberazione, regime fiscale.</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IPOTESI: prassi 10%; il testo estratto dell'avviso non riporta la percentuale, verificarla</t>
+          <t>Dato: avviso, sezione F (cauzione 10% del prezzo offerto)</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Dato: perizia (2 anni di ordinarie 6.700 + straordinarie deliberate 2.650)</t>
+          <t>IPOTESI prudenziale: importi che la perizia detrae dal valore (2 anni di ordinarie 6.700 + straordinarie 2.650); gli insoluti veri si chiedono all'amministratore</t>
         </is>
       </c>
     </row>
@@ -7167,7 +7167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -7331,7 +7331,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cauzione: percentuale da verificare nell'avviso</t>
+          <t>Fascia di rispetto dell'elettrodotto (avviso e perizia)</t>
         </is>
       </c>
       <c r="B18" s="14" t="n">
@@ -7341,32 +7341,42 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aliquota di registro e trattamento IVA da confermare col parere fiscale</t>
+          <t>Impianti senza certificazioni, APE classe F (perizia)</t>
         </is>
       </c>
       <c r="B19" s="14" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Errori totali</t>
-        </is>
-      </c>
-      <c r="B21" s="7">
-        <f>SUM(B3:B10)</f>
-        <v/>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Aliquota di registro e trattamento IVA da confermare col parere fiscale</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
+          <t>Errori totali</t>
+        </is>
+      </c>
+      <c r="B22" s="7">
+        <f>SUM(B3:B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
           <t>Avvisi totali</t>
         </is>
       </c>
-      <c r="B22" s="7">
-        <f>SUM(B13:B19)</f>
+      <c r="B23" s="7">
+        <f>SUM(B13:B20)</f>
         <v/>
       </c>
     </row>

</xml_diff>